<commit_message>
Add Time Extension service request automation; support-screen updates
Fixes a stale UI-close-button wait that silently broke the Start/Stop
Time Extension approve flow, corrects test data/assertions against
live app behavior, and adds Corporate Service Request, Child Pause,
and Recent Customer Request grid support used across these suites.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testData/input_UserRights.xlsx
+++ b/testData/input_UserRights.xlsx
@@ -397,7 +397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.515625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="5" min="1" max="1"/>
@@ -470,6 +470,23 @@
       <c r="C4" s="5" t="inlineStr">
         <is>
           <t>View_Account_Statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Varsha Jha</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Corporate Account Statement</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tieup_SPOC_Access</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Transport 1way and 2way
</commit_message>
<xml_diff>
--- a/testData/input_UserRights.xlsx
+++ b/testData/input_UserRights.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="UserRights" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UserRights" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -397,7 +397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.515625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="5" min="1" max="1"/>
@@ -474,19 +474,36 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Varsha Jha</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Corporate Account Statement</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Tieup_SPOC_Access</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nidhi Chaturvedi</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Raise_Support_Request</t>
         </is>
       </c>
     </row>

</xml_diff>